<commit_message>
feat(pricing): taxas TikTok Shop no motor e no simulador
- tiktok_pricing_engine.py: comissão por faixa (10% + R$4 < R$50; 6% + R$6 >= R$50),
  SFP 6% e transação 3% sempre cobrados (validado no extrato AKG de 05/10/2026);
  isenção de novo vendedor zera só a comissão; busca via Partner API Finance
  quando houver credenciais (fallback para a tabela)
- pricing_engine_real.py: canais "TikTok Shop" e "TikTok Shop AKG" calculados
  sem depender de regra cadastrada, com resolução da faixa em R$50
- app.py: alias dos canais TikTok e fonte de taxa em /taxas/status
- simulador: selo TikTok; planilha V8 com linhas TikTok e imposto do bloco Margem

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Simulador_2026_V8_beta.xlsx
+++ b/Simulador_2026_V8_beta.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabio\Downloads\shinsei-pricing\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fabio\Downloads\shinsei_pricing\shinsei_pricing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ED7D005-3185-40F6-AA2C-1F2DF152007D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B5D600D6-30F7-450C-BA0C-AC3A0719B187}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" tabRatio="472" activeTab="3" xr2:uid="{889A097E-C5EB-4328-803A-460C29B34FEE}"/>
+    <workbookView xWindow="2640" yWindow="2220" windowWidth="21600" windowHeight="11100" tabRatio="472" activeTab="3" xr2:uid="{889A097E-C5EB-4328-803A-460C29B34FEE}"/>
   </bookViews>
   <sheets>
     <sheet name="Aba1" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="597" uniqueCount="49">
   <si>
     <t>Valor</t>
   </si>
@@ -184,6 +184,15 @@
   <si>
     <t>M.D.C</t>
   </si>
+  <si>
+    <t>TikTok Shop</t>
+  </si>
+  <si>
+    <t>TikTok: comissão 10% + SFP 6% + transação 3% + R$4/item. Na isenção de novo vendedor, trocar 0,1 por 0</t>
+  </si>
+  <si>
+    <t>TikTok: comissão 6% + SFP 6% + transação 3% + R$6/item. Na isenção de novo vendedor, trocar o primeiro 0,06 por 0</t>
+  </si>
 </sst>
 </file>
 
@@ -193,7 +202,7 @@
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="43" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="166" formatCode="0.0000"/>
+    <numFmt numFmtId="165" formatCode="0.0000"/>
   </numFmts>
   <fonts count="9">
     <font>
@@ -700,7 +709,7 @@
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="122">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -970,22 +979,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
@@ -1004,6 +997,16 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
       <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyProtection="1">
+      <protection locked="0"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
@@ -1097,15 +1100,9 @@
       <alignment horizontal="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="2" applyFont="1" applyProtection="1">
-      <protection locked="0"/>
+      <protection hidden="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -1571,78 +1568,78 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{506FB158-B15D-4A85-A68E-5C19D1A3CC70}">
-  <dimension ref="A1:Q22"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="A1:Q23"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="16.08984375" style="34" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="10.81640625" style="38" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="8.7265625" style="34"/>
-    <col min="4" max="4" width="12.6328125" style="34" customWidth="1"/>
-    <col min="5" max="5" width="22.26953125" style="34" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="12.26953125" style="34" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="10.81640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="9.7265625" style="37" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="13.81640625" style="37" customWidth="1"/>
-    <col min="11" max="11" width="10.81640625" style="37" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="13.453125" style="37" customWidth="1"/>
-    <col min="13" max="13" width="16.6328125" style="39" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" style="34" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.85546875" style="38" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" style="34"/>
+    <col min="4" max="4" width="12.5703125" style="34" customWidth="1"/>
+    <col min="5" max="5" width="22.28515625" style="34" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="12.28515625" style="34" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.85546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.7109375" style="37" hidden="1" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" style="37" customWidth="1"/>
+    <col min="11" max="11" width="10.85546875" style="37" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="13.42578125" style="37" customWidth="1"/>
+    <col min="13" max="13" width="16.5703125" style="39" customWidth="1"/>
     <col min="14" max="14" width="0" style="34" hidden="1" customWidth="1"/>
-    <col min="15" max="15" width="8.7265625" style="34"/>
-    <col min="16" max="16" width="10.81640625" style="34" bestFit="1" customWidth="1"/>
-    <col min="17" max="16384" width="8.7265625" style="34"/>
+    <col min="15" max="15" width="8.7109375" style="34"/>
+    <col min="16" max="16" width="10.85546875" style="34" bestFit="1" customWidth="1"/>
+    <col min="17" max="16384" width="8.7109375" style="34"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" ht="26.5" thickBot="1">
-      <c r="A1" s="102" t="s">
+    <row r="1" spans="1:17" ht="27" thickBot="1">
+      <c r="A1" s="101" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="103"/>
-      <c r="C1" s="103"/>
-      <c r="D1" s="103"/>
-      <c r="E1" s="103"/>
-      <c r="F1" s="103"/>
-      <c r="G1" s="103"/>
-      <c r="H1" s="103"/>
-      <c r="I1" s="103"/>
-      <c r="J1" s="103"/>
-      <c r="K1" s="103"/>
-      <c r="L1" s="103"/>
-      <c r="M1" s="104"/>
-    </row>
-    <row r="2" spans="1:17" ht="21.5" thickBot="1">
-      <c r="A2" s="110" t="s">
+      <c r="B1" s="102"/>
+      <c r="C1" s="102"/>
+      <c r="D1" s="102"/>
+      <c r="E1" s="102"/>
+      <c r="F1" s="102"/>
+      <c r="G1" s="102"/>
+      <c r="H1" s="102"/>
+      <c r="I1" s="102"/>
+      <c r="J1" s="102"/>
+      <c r="K1" s="102"/>
+      <c r="L1" s="102"/>
+      <c r="M1" s="103"/>
+    </row>
+    <row r="2" spans="1:17" ht="21.75" thickBot="1">
+      <c r="A2" s="109" t="s">
         <v>19</v>
       </c>
-      <c r="B2" s="111"/>
-      <c r="C2" s="100" t="s">
+      <c r="B2" s="110"/>
+      <c r="C2" s="99" t="s">
         <v>39</v>
       </c>
-      <c r="D2" s="101"/>
-      <c r="E2" s="112" t="s">
+      <c r="D2" s="100"/>
+      <c r="E2" s="111" t="s">
         <v>20</v>
       </c>
-      <c r="F2" s="112"/>
-      <c r="G2" s="111"/>
-      <c r="H2" s="100" t="s">
+      <c r="F2" s="111"/>
+      <c r="G2" s="110"/>
+      <c r="H2" s="99" t="s">
         <v>40</v>
       </c>
-      <c r="I2" s="113"/>
-      <c r="J2" s="113"/>
-      <c r="K2" s="114"/>
-      <c r="L2" s="100" t="s">
+      <c r="I2" s="112"/>
+      <c r="J2" s="112"/>
+      <c r="K2" s="113"/>
+      <c r="L2" s="99" t="s">
         <v>44</v>
       </c>
-      <c r="M2" s="115"/>
-    </row>
-    <row r="3" spans="1:17" ht="16">
+      <c r="M2" s="114"/>
+    </row>
+    <row r="3" spans="1:17" ht="15.75">
       <c r="A3" s="41" t="s">
         <v>21</v>
       </c>
       <c r="B3" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C3" s="96"/>
-      <c r="D3" s="97"/>
+      <c r="C3" s="95"/>
+      <c r="D3" s="96"/>
       <c r="E3" s="43" t="s">
         <v>1</v>
       </c>
@@ -1662,20 +1659,20 @@
       <c r="K3" s="48" t="s">
         <v>43</v>
       </c>
-      <c r="L3" s="108" t="s">
+      <c r="L3" s="107" t="s">
         <v>45</v>
       </c>
-      <c r="M3" s="109"/>
-    </row>
-    <row r="4" spans="1:17" ht="16">
+      <c r="M3" s="108"/>
+    </row>
+    <row r="4" spans="1:17" ht="15.75">
       <c r="A4" s="41" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="26">
         <v>80</v>
       </c>
-      <c r="C4" s="96"/>
-      <c r="D4" s="97"/>
+      <c r="C4" s="95"/>
+      <c r="D4" s="96"/>
       <c r="E4" s="49" t="s">
         <v>16</v>
       </c>
@@ -1716,15 +1713,15 @@
         <v>6.2650000000000006</v>
       </c>
     </row>
-    <row r="5" spans="1:17" ht="16">
+    <row r="5" spans="1:17" ht="15.75">
       <c r="A5" s="41" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="26">
         <v>1.5</v>
       </c>
-      <c r="C5" s="96"/>
-      <c r="D5" s="97"/>
+      <c r="C5" s="95"/>
+      <c r="D5" s="96"/>
       <c r="E5" s="49" t="s">
         <v>13</v>
       </c>
@@ -1762,15 +1759,15 @@
         <v>6.6615189873417728</v>
       </c>
     </row>
-    <row r="6" spans="1:17" ht="16">
+    <row r="6" spans="1:17" ht="15.75">
       <c r="A6" s="41" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="27">
         <v>0.3</v>
       </c>
-      <c r="C6" s="96"/>
-      <c r="D6" s="97"/>
+      <c r="C6" s="95"/>
+      <c r="D6" s="96"/>
       <c r="E6" s="56" t="s">
         <v>14</v>
       </c>
@@ -1808,15 +1805,15 @@
         <v>6.7576315789473691</v>
       </c>
     </row>
-    <row r="7" spans="1:17" ht="16">
+    <row r="7" spans="1:17" ht="15.75">
       <c r="A7" s="41" t="s">
         <v>30</v>
       </c>
       <c r="B7" s="28">
         <v>1.33</v>
       </c>
-      <c r="C7" s="96"/>
-      <c r="D7" s="97"/>
+      <c r="C7" s="95"/>
+      <c r="D7" s="96"/>
       <c r="E7" s="64" t="s">
         <v>17</v>
       </c>
@@ -1855,15 +1852,15 @@
       </c>
       <c r="P7" s="40"/>
     </row>
-    <row r="8" spans="1:17" ht="16">
+    <row r="8" spans="1:17" ht="15.75">
       <c r="A8" s="41" t="s">
         <v>31</v>
       </c>
       <c r="B8" s="29">
         <v>0.04</v>
       </c>
-      <c r="C8" s="96"/>
-      <c r="D8" s="97"/>
+      <c r="C8" s="95"/>
+      <c r="D8" s="96"/>
       <c r="E8" s="43" t="s">
         <v>11</v>
       </c>
@@ -1908,8 +1905,8 @@
       <c r="B9" s="36">
         <v>1</v>
       </c>
-      <c r="C9" s="98"/>
-      <c r="D9" s="99"/>
+      <c r="C9" s="97"/>
+      <c r="D9" s="98"/>
       <c r="E9" s="78" t="s">
         <v>35</v>
       </c>
@@ -1947,111 +1944,137 @@
         <v>5.259540229885058</v>
       </c>
     </row>
-    <row r="10" spans="1:17" ht="15" thickBot="1">
-      <c r="A10" s="86"/>
-      <c r="B10" s="87"/>
+    <row r="10" spans="1:17" ht="16.5" thickBot="1">
+      <c r="A10" s="77"/>
+      <c r="B10" s="36"/>
       <c r="C10" s="86"/>
       <c r="D10" s="86"/>
-      <c r="E10" s="86"/>
-      <c r="F10" s="86"/>
-      <c r="G10" s="86"/>
-      <c r="H10" s="88"/>
-      <c r="I10" s="89"/>
-      <c r="J10" s="88"/>
-      <c r="K10" s="88"/>
-      <c r="L10" s="88"/>
-      <c r="M10" s="90"/>
-      <c r="N10" s="35"/>
-    </row>
-    <row r="11" spans="1:17" ht="26.5" thickBot="1">
-      <c r="A11" s="105" t="s">
+      <c r="E10" s="78" t="s">
+        <v>46</v>
+      </c>
+      <c r="F10" s="79">
+        <f>'Aba3'!G8</f>
+        <v>141.22839506172841</v>
+      </c>
+      <c r="G10" s="80">
+        <f>'Aba3'!L8</f>
+        <v>114.04413580246914</v>
+      </c>
+      <c r="H10" s="81">
+        <f>$I$4</f>
+        <v>80</v>
+      </c>
+      <c r="I10" s="79"/>
+      <c r="J10" s="82">
+        <f>F10-G10</f>
+        <v>27.184259259259264</v>
+      </c>
+      <c r="K10" s="83">
+        <f>H10+J10</f>
+        <v>107.18425925925926</v>
+      </c>
+      <c r="L10" s="84">
+        <f>F10-H10-J10-N10-$B$5</f>
+        <v>26.895000000000007</v>
+      </c>
+      <c r="M10" s="85">
+        <f>L10/F10</f>
+        <v>0.1904362078762184</v>
+      </c>
+      <c r="N10" s="35">
+        <f>$B$8*F10</f>
+        <v>5.6491358024691367</v>
+      </c>
+    </row>
+    <row r="11" spans="1:17" ht="27" thickBot="1">
+      <c r="A11" s="104" t="s">
         <v>32</v>
       </c>
-      <c r="B11" s="106"/>
-      <c r="C11" s="106"/>
-      <c r="D11" s="106"/>
-      <c r="E11" s="106"/>
-      <c r="F11" s="106"/>
-      <c r="G11" s="106"/>
-      <c r="H11" s="106"/>
-      <c r="I11" s="106"/>
-      <c r="J11" s="106"/>
-      <c r="K11" s="106"/>
-      <c r="L11" s="106"/>
-      <c r="M11" s="107"/>
+      <c r="B11" s="105"/>
+      <c r="C11" s="105"/>
+      <c r="D11" s="105"/>
+      <c r="E11" s="105"/>
+      <c r="F11" s="105"/>
+      <c r="G11" s="105"/>
+      <c r="H11" s="105"/>
+      <c r="I11" s="105"/>
+      <c r="J11" s="105"/>
+      <c r="K11" s="105"/>
+      <c r="L11" s="105"/>
+      <c r="M11" s="106"/>
       <c r="N11" s="35"/>
     </row>
-    <row r="12" spans="1:17" ht="21.5" thickBot="1">
-      <c r="A12" s="110" t="s">
+    <row r="12" spans="1:17" ht="21.75" thickBot="1">
+      <c r="A12" s="109" t="s">
         <v>19</v>
       </c>
-      <c r="B12" s="111"/>
-      <c r="C12" s="100" t="str">
+      <c r="B12" s="110"/>
+      <c r="C12" s="99" t="str">
         <f>C2</f>
         <v>Calculadora</v>
       </c>
-      <c r="D12" s="101"/>
-      <c r="E12" s="112" t="s">
+      <c r="D12" s="100"/>
+      <c r="E12" s="111" t="s">
         <v>20</v>
       </c>
-      <c r="F12" s="112"/>
-      <c r="G12" s="111"/>
-      <c r="H12" s="116" t="s">
+      <c r="F12" s="111"/>
+      <c r="G12" s="110"/>
+      <c r="H12" s="115" t="s">
         <v>40</v>
       </c>
-      <c r="I12" s="117"/>
-      <c r="J12" s="117"/>
-      <c r="K12" s="118"/>
-      <c r="L12" s="100" t="s">
+      <c r="I12" s="116"/>
+      <c r="J12" s="116"/>
+      <c r="K12" s="117"/>
+      <c r="L12" s="99" t="s">
         <v>44</v>
       </c>
-      <c r="M12" s="115"/>
+      <c r="M12" s="114"/>
       <c r="N12" s="35"/>
     </row>
-    <row r="13" spans="1:17" ht="16">
+    <row r="13" spans="1:17" ht="15.75">
       <c r="A13" s="41" t="s">
         <v>21</v>
       </c>
       <c r="B13" s="42" t="s">
         <v>0</v>
       </c>
-      <c r="C13" s="96"/>
-      <c r="D13" s="97"/>
+      <c r="C13" s="95"/>
+      <c r="D13" s="96"/>
       <c r="E13" s="43" t="s">
         <v>1</v>
       </c>
       <c r="F13" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="G13" s="91" t="s">
+      <c r="G13" s="87" t="s">
         <v>33</v>
       </c>
-      <c r="H13" s="92" t="s">
+      <c r="H13" s="88" t="s">
         <v>41</v>
       </c>
-      <c r="I13" s="93"/>
-      <c r="J13" s="94" t="s">
+      <c r="I13" s="89"/>
+      <c r="J13" s="90" t="s">
         <v>42</v>
       </c>
-      <c r="K13" s="95" t="s">
+      <c r="K13" s="91" t="s">
         <v>43</v>
       </c>
-      <c r="L13" s="108" t="str">
+      <c r="L13" s="107" t="str">
         <f>L3</f>
         <v>M.D.C</v>
       </c>
-      <c r="M13" s="109"/>
+      <c r="M13" s="108"/>
       <c r="N13" s="35"/>
     </row>
-    <row r="14" spans="1:17" ht="16">
+    <row r="14" spans="1:17" ht="15.75">
       <c r="A14" s="41" t="s">
         <v>2</v>
       </c>
       <c r="B14" s="30">
         <v>80</v>
       </c>
-      <c r="C14" s="96"/>
-      <c r="D14" s="97"/>
+      <c r="C14" s="95"/>
+      <c r="D14" s="96"/>
       <c r="E14" s="49" t="s">
         <v>16</v>
       </c>
@@ -2085,23 +2108,23 @@
         <v>0.29999999999999993</v>
       </c>
       <c r="N14" s="35">
-        <f t="shared" si="4"/>
+        <f>$B$18*F14</f>
         <v>7.753333333333333</v>
       </c>
-      <c r="O14" s="120">
+      <c r="O14" s="93">
         <f>L14/F14</f>
         <v>0.29999999999999993</v>
       </c>
       <c r="P14" s="35">
-        <f>$F$20-L14</f>
-        <v>133.77164953283247</v>
-      </c>
-      <c r="Q14" s="121">
+        <f>$F$21-L14</f>
+        <v>130.86407494971073</v>
+      </c>
+      <c r="Q14" s="94">
         <f t="shared" ref="Q14:Q19" si="7">P14/F14</f>
-        <v>0.69013748684178411</v>
-      </c>
-    </row>
-    <row r="15" spans="1:17" ht="16">
+        <v>0.67513710206213629</v>
+      </c>
+    </row>
+    <row r="15" spans="1:17" ht="15.75">
       <c r="A15" s="41" t="s">
         <v>3</v>
       </c>
@@ -2109,8 +2132,8 @@
         <f>B5</f>
         <v>1.5</v>
       </c>
-      <c r="C15" s="96"/>
-      <c r="D15" s="97"/>
+      <c r="C15" s="95"/>
+      <c r="D15" s="96"/>
       <c r="E15" s="49" t="s">
         <v>13</v>
       </c>
@@ -2144,23 +2167,23 @@
         <v>0.3</v>
       </c>
       <c r="N15" s="35">
-        <f t="shared" si="4"/>
+        <f>$B$18*F15</f>
         <v>8.8138775510204095</v>
       </c>
-      <c r="O15" s="120">
+      <c r="O15" s="93">
         <f t="shared" ref="O15:O19" si="10">L15/F15</f>
         <v>0.3</v>
       </c>
       <c r="P15" s="35">
-        <f t="shared" ref="P15:P19" si="11">$F$20-L15</f>
-        <v>125.81756790017938</v>
-      </c>
-      <c r="Q15" s="121">
+        <f t="shared" ref="P15:P19" si="11">$F$21-L15</f>
+        <v>122.90999331705764</v>
+      </c>
+      <c r="Q15" s="94">
         <f t="shared" si="7"/>
-        <v>0.57099757591078903</v>
-      </c>
-    </row>
-    <row r="16" spans="1:17" ht="16">
+        <v>0.55780213693950398</v>
+      </c>
+    </row>
+    <row r="16" spans="1:17" ht="15.75">
       <c r="A16" s="41" t="s">
         <v>4</v>
       </c>
@@ -2168,8 +2191,8 @@
         <f>B6</f>
         <v>0.3</v>
       </c>
-      <c r="C16" s="96"/>
-      <c r="D16" s="97"/>
+      <c r="C16" s="95"/>
+      <c r="D16" s="96"/>
       <c r="E16" s="56" t="s">
         <v>14</v>
       </c>
@@ -2203,31 +2226,31 @@
         <v>0.3000000000000001</v>
       </c>
       <c r="N16" s="35">
-        <f t="shared" si="4"/>
+        <f>$B$18*F16</f>
         <v>8.8260869565217401</v>
       </c>
-      <c r="O16" s="120">
+      <c r="O16" s="93">
         <f t="shared" si="10"/>
         <v>0.3000000000000001</v>
       </c>
       <c r="P16" s="35">
         <f t="shared" si="11"/>
-        <v>125.72599735891937</v>
-      </c>
-      <c r="Q16" s="121">
+        <v>122.81842277579763</v>
+      </c>
+      <c r="Q16" s="94">
         <f t="shared" si="7"/>
-        <v>0.56979269739017646</v>
-      </c>
-    </row>
-    <row r="17" spans="1:17" ht="16">
+        <v>0.55661551208735871</v>
+      </c>
+    </row>
+    <row r="17" spans="1:17" ht="15.75">
       <c r="A17" s="41" t="s">
         <v>32</v>
       </c>
       <c r="B17" s="29">
         <v>0.3</v>
       </c>
-      <c r="C17" s="96"/>
-      <c r="D17" s="97"/>
+      <c r="C17" s="95"/>
+      <c r="D17" s="96"/>
       <c r="E17" s="64" t="s">
         <v>17</v>
       </c>
@@ -2261,23 +2284,23 @@
         <v>0.29999999999999982</v>
       </c>
       <c r="N17" s="35">
-        <f t="shared" si="4"/>
+        <f>$B$18*F17</f>
         <v>7.60754716981132</v>
       </c>
-      <c r="O17" s="120">
+      <c r="O17" s="93">
         <f t="shared" si="10"/>
         <v>0.29999999999999982</v>
       </c>
       <c r="P17" s="35">
         <f t="shared" si="11"/>
-        <v>134.86504575924758</v>
-      </c>
-      <c r="Q17" s="121">
+        <v>131.95747117612584</v>
+      </c>
+      <c r="Q17" s="94">
         <f t="shared" si="7"/>
-        <v>0.7091118477420757</v>
-      </c>
-    </row>
-    <row r="18" spans="1:17" ht="16">
+        <v>0.69382400519193155</v>
+      </c>
+    </row>
+    <row r="18" spans="1:17" ht="15.75">
       <c r="A18" s="41" t="s">
         <v>31</v>
       </c>
@@ -2285,8 +2308,8 @@
         <f>B8</f>
         <v>0.04</v>
       </c>
-      <c r="C18" s="96"/>
-      <c r="D18" s="97"/>
+      <c r="C18" s="95"/>
+      <c r="D18" s="96"/>
       <c r="E18" s="43" t="s">
         <v>11</v>
       </c>
@@ -2320,20 +2343,20 @@
         <v>0.29999999999999993</v>
       </c>
       <c r="N18" s="35">
-        <f t="shared" si="4"/>
+        <f>$B$18*F18</f>
         <v>6.92</v>
       </c>
-      <c r="O18" s="120">
+      <c r="O18" s="93">
         <f t="shared" si="10"/>
         <v>0.29999999999999993</v>
       </c>
       <c r="P18" s="35">
         <f t="shared" si="11"/>
-        <v>140.02164953283244</v>
-      </c>
-      <c r="Q18" s="121">
+        <v>137.1140749497107</v>
+      </c>
+      <c r="Q18" s="94">
         <f t="shared" si="7"/>
-        <v>0.80937369672157478</v>
+        <v>0.79256690722376122</v>
       </c>
     </row>
     <row r="19" spans="1:17" ht="16.5" thickBot="1">
@@ -2345,8 +2368,8 @@
         <f>B9</f>
         <v>1</v>
       </c>
-      <c r="C19" s="98"/>
-      <c r="D19" s="99"/>
+      <c r="C19" s="97"/>
+      <c r="D19" s="98"/>
       <c r="E19" s="78" t="s">
         <v>35</v>
       </c>
@@ -2380,43 +2403,97 @@
         <v>0.29999999999999988</v>
       </c>
       <c r="N19" s="35">
-        <f t="shared" si="4"/>
+        <f>$B$18*F19</f>
         <v>6.140350877192982</v>
       </c>
-      <c r="O19" s="120">
+      <c r="O19" s="93">
         <f t="shared" si="10"/>
         <v>0.29999999999999988</v>
       </c>
       <c r="P19" s="35">
         <f t="shared" si="11"/>
-        <v>145.86901795388511</v>
-      </c>
-      <c r="Q19" s="121">
+        <v>142.96144337076336</v>
+      </c>
+      <c r="Q19" s="94">
         <f t="shared" si="7"/>
-        <v>0.95023245981388016</v>
-      </c>
-    </row>
-    <row r="20" spans="1:17">
-      <c r="F20" s="35">
-        <f>AVERAGE(F14:F19)</f>
-        <v>191.92164953283245</v>
-      </c>
-      <c r="L20" s="119">
-        <f>AVERAGE(L14:L19)</f>
-        <v>57.576494859849724</v>
+        <v>0.93129168824383002</v>
+      </c>
+    </row>
+    <row r="20" spans="1:17" ht="16.5" thickBot="1">
+      <c r="A20" s="77"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="118"/>
+      <c r="D20" s="118"/>
+      <c r="E20" s="78" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="79">
+        <f>'Aba3'!G19</f>
+        <v>171.56862745098039</v>
+      </c>
+      <c r="G20" s="82">
+        <f>'Aba3'!L19</f>
+        <v>139.83333333333331</v>
+      </c>
+      <c r="H20" s="81">
+        <f>$I$4</f>
+        <v>80</v>
+      </c>
+      <c r="I20" s="79"/>
+      <c r="J20" s="82">
+        <f>F20-G20</f>
+        <v>31.735294117647072</v>
+      </c>
+      <c r="K20" s="82">
+        <f>H20+J20</f>
+        <v>111.73529411764707</v>
+      </c>
+      <c r="L20" s="81">
+        <f>F20-H20-J20-N20-$B$5</f>
+        <v>51.470588235294102</v>
+      </c>
+      <c r="M20" s="85">
+        <f>L20/F20</f>
+        <v>0.29999999999999993</v>
+      </c>
+      <c r="N20" s="35">
+        <f>$B$18*F20</f>
+        <v>6.8627450980392153</v>
+      </c>
+      <c r="O20" s="93">
+        <f>L20/F20</f>
+        <v>0.29999999999999993</v>
       </c>
       <c r="P20" s="35">
-        <f>AVERAGE(P14:P19)</f>
-        <v>134.34515467298272</v>
-      </c>
-      <c r="Q20" s="121">
+        <f>$F$21-L20</f>
+        <v>137.54348671441659</v>
+      </c>
+      <c r="Q20" s="94">
         <f>P20/F20</f>
+        <v>0.80168203684974237</v>
+      </c>
+    </row>
+    <row r="21" spans="1:17">
+      <c r="F21" s="35">
+        <f>AVERAGE(F14:F20)</f>
+        <v>189.0140749497107</v>
+      </c>
+      <c r="L21" s="92">
+        <f>AVERAGE(L14:L20)</f>
+        <v>56.704222484913203</v>
+      </c>
+      <c r="P21" s="35">
+        <f>AVERAGE(P14:P20)</f>
+        <v>132.3098524647975</v>
+      </c>
+      <c r="Q21" s="94">
+        <f>P21/F21</f>
         <v>0.70000000000000007</v>
       </c>
     </row>
-    <row r="22" spans="1:17">
-      <c r="L22" s="37">
-        <f>L20/F20</f>
+    <row r="23" spans="1:17">
+      <c r="L23" s="37">
+        <f>L21/F21</f>
         <v>0.29999999999999993</v>
       </c>
     </row>
@@ -2448,17 +2525,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{36EBE32C-FB8F-4769-9B9E-E76874140199}">
-  <dimension ref="A1:M496"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="A1:M498"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="20" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="11.1796875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="18.90625" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="10.08984375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.90625" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.90625" customWidth="1"/>
+    <col min="5" max="5" width="18.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="10.140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.85546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9">
@@ -14925,6 +15002,66 @@
       </c>
       <c r="H496" s="1">
         <v>0.5</v>
+      </c>
+    </row>
+    <row r="497" spans="1:9">
+      <c r="A497" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B497" s="1">
+        <v>0</v>
+      </c>
+      <c r="C497" s="1">
+        <v>9999999</v>
+      </c>
+      <c r="D497" s="20">
+        <v>0.01</v>
+      </c>
+      <c r="E497" s="20">
+        <v>49.99</v>
+      </c>
+      <c r="F497" s="3">
+        <v>4</v>
+      </c>
+      <c r="G497" s="3">
+        <v>0</v>
+      </c>
+      <c r="H497" s="1">
+        <f>0.1+0.06+0.03</f>
+        <v>0.19</v>
+      </c>
+      <c r="I497" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="498" spans="1:9">
+      <c r="A498" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B498" s="1">
+        <v>0</v>
+      </c>
+      <c r="C498" s="1">
+        <v>9999999</v>
+      </c>
+      <c r="D498" s="20">
+        <v>50</v>
+      </c>
+      <c r="E498" s="20">
+        <v>999999999</v>
+      </c>
+      <c r="F498" s="3">
+        <v>6</v>
+      </c>
+      <c r="G498" s="3">
+        <v>0</v>
+      </c>
+      <c r="H498" s="1">
+        <f>0.06+0.06+0.03</f>
+        <v>0.15</v>
+      </c>
+      <c r="I498" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -14935,7 +15072,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D4D601ED-C77A-4CE4-911B-76C196C5EAE7}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <sheetData/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -14943,26 +15080,26 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B4F2AA4B-431D-46CE-BBB9-45509BCC6344}">
-  <dimension ref="A1:O18"/>
-  <sheetFormatPr defaultRowHeight="14.5"/>
+  <dimension ref="A1:O19"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="31.08984375" style="4" customWidth="1"/>
-    <col min="2" max="2" width="9.26953125" style="4" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="7.81640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="31.140625" style="4" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" style="4" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.85546875" style="4" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="9" style="4" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.6328125" style="4" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="10.81640625" style="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="13.1796875" style="4" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="8.7265625" style="4"/>
-    <col min="10" max="10" width="11.08984375" style="4" customWidth="1"/>
+    <col min="5" max="5" width="10.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.5703125" style="4" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.85546875" style="4" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="13.140625" style="4" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="8.7109375" style="4"/>
+    <col min="10" max="10" width="11.140625" style="4" customWidth="1"/>
     <col min="11" max="11" width="16" style="4" customWidth="1"/>
-    <col min="12" max="12" width="10.90625" style="4" customWidth="1"/>
-    <col min="13" max="15" width="9.7265625" style="4" bestFit="1" customWidth="1"/>
-    <col min="16" max="16384" width="8.7265625" style="4"/>
+    <col min="12" max="12" width="10.85546875" style="4" customWidth="1"/>
+    <col min="13" max="15" width="9.7109375" style="4" bestFit="1" customWidth="1"/>
+    <col min="16" max="16384" width="8.7109375" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" ht="28">
+    <row r="1" spans="1:15" ht="30">
       <c r="A1" s="10" t="s">
         <v>1</v>
       </c>
@@ -15284,7 +15421,50 @@
       </c>
     </row>
     <row r="8" spans="1:15">
-      <c r="H8" s="23"/>
+      <c r="A8" s="24" t="s">
+        <v>46</v>
+      </c>
+      <c r="B8" s="22">
+        <f>'Aba1'!$I$4+'Aba1'!$B$5</f>
+        <v>81.5</v>
+      </c>
+      <c r="C8" s="12">
+        <f>IF(((B8*F8)+'Aba2'!$F$497+E8)/(1-'Aba2'!$H$497-'Aba1'!$B$8)&lt;'Aba2'!$D$498,'Aba2'!$H$497,'Aba2'!$H$498)</f>
+        <v>0.15</v>
+      </c>
+      <c r="D8" s="21">
+        <f>IF(((B8*F8)+'Aba2'!$F$497+E8)/(1-'Aba2'!$H$497-'Aba1'!$B$8)&lt;'Aba2'!$D$498,'Aba2'!$F$497,'Aba2'!$F$498)</f>
+        <v>6</v>
+      </c>
+      <c r="E8" s="21">
+        <f>'Aba2'!$G$497</f>
+        <v>0</v>
+      </c>
+      <c r="F8" s="14">
+        <f>'Aba1'!$B$7</f>
+        <v>1.33</v>
+      </c>
+      <c r="G8" s="21">
+        <f>MAX(((B8*F8)+D8+E8)/(1-C8-'Aba1'!$B$8),IF(C8='Aba2'!$H$498,'Aba2'!$D$498,0))</f>
+        <v>141.22839506172841</v>
+      </c>
+      <c r="H8" s="22">
+        <f>G8-(B8+D8+E8+(G8*C8)+(G8*'Aba1'!$B$8))</f>
+        <v>26.89500000000001</v>
+      </c>
+      <c r="I8" s="16">
+        <f>H8/B8</f>
+        <v>0.33000000000000013</v>
+      </c>
+      <c r="J8" s="17">
+        <f>G8*C8</f>
+        <v>21.18425925925926</v>
+      </c>
+      <c r="K8" s="17"/>
+      <c r="L8" s="18">
+        <f>G8-D8-E8-J8</f>
+        <v>114.04413580246914</v>
+      </c>
     </row>
     <row r="9" spans="1:15">
       <c r="H9" s="23"/>
@@ -15295,7 +15475,7 @@
     <row r="11" spans="1:15">
       <c r="H11" s="23"/>
     </row>
-    <row r="12" spans="1:15" ht="28">
+    <row r="12" spans="1:15" ht="45">
       <c r="A12" s="6" t="s">
         <v>1</v>
       </c>
@@ -15358,7 +15538,7 @@
         <v>193.83333333333331</v>
       </c>
       <c r="H13" s="22">
-        <f>G13-(B13+D13+E13+(G13*C13)+(G13*'Aba1'!$B$8))</f>
+        <f>G13-(B13+D13+E13+(G13*C13)+(G13*'Aba1'!$B$18))</f>
         <v>58.149999999999977</v>
       </c>
       <c r="I13" s="16">
@@ -15402,7 +15582,7 @@
         <v>220.34693877551021</v>
       </c>
       <c r="H14" s="22">
-        <f>G14-(B14+D14+E14+(G14*C14)+(G14*'Aba1'!$B$8))</f>
+        <f>G14-(B14+D14+E14+(G14*C14)+(G14*'Aba1'!$B$18))</f>
         <v>66.104081632653077</v>
       </c>
       <c r="I14" s="16">
@@ -15447,7 +15627,7 @@
         <v>220.6521739130435</v>
       </c>
       <c r="H15" s="22">
-        <f>G15-(B15+D15+E15+(G15*C15)+(G15*'Aba1'!$B$8))</f>
+        <f>G15-(B15+D15+E15+(G15*C15)+(G15*'Aba1'!$B$18))</f>
         <v>66.195652173913061</v>
       </c>
       <c r="I15" s="16">
@@ -15492,7 +15672,7 @@
         <v>190.188679245283</v>
       </c>
       <c r="H16" s="22">
-        <f>G16-(B16+D16+E16+(G16*C16)+(G16*'Aba1'!$B$8))</f>
+        <f>G16-(B16+D16+E16+(G16*C16)+(G16*'Aba1'!$B$18))</f>
         <v>57.056603773584897</v>
       </c>
       <c r="I16" s="16">
@@ -15537,7 +15717,7 @@
         <v>173</v>
       </c>
       <c r="H17" s="22">
-        <f>G17-(B17+D17+E17+(G17*C17)+(G17*'Aba1'!$B$8))</f>
+        <f>G17-(B17+D17+E17+(G17*C17)+(G17*'Aba1'!$B$18))</f>
         <v>51.899999999999991</v>
       </c>
       <c r="I17" s="16">
@@ -15583,7 +15763,7 @@
         <v>153.50877192982455</v>
       </c>
       <c r="H18" s="22">
-        <f>G18-(B18+D18+E18+(G18*C18)+(G18*'Aba1'!$B$8))</f>
+        <f>G18-(B18+D18+E18+(G18*C18)+(G18*'Aba1'!$B$18))</f>
         <v>46.052631578947356</v>
       </c>
       <c r="I18" s="16">
@@ -15600,6 +15780,52 @@
         <v>133.69298245614033</v>
       </c>
     </row>
+    <row r="19" spans="1:12">
+      <c r="A19" s="7" t="s">
+        <v>46</v>
+      </c>
+      <c r="B19" s="19">
+        <f>'Aba1'!$I$4+'Aba1'!$B$15</f>
+        <v>81.5</v>
+      </c>
+      <c r="C19" s="8">
+        <f>IF((B19+'Aba2'!$F$497+E19)/(1-('Aba2'!$H$497+'Aba1'!$B$17+'Aba1'!$B$18))&lt;'Aba2'!$D$498,'Aba2'!$H$497,'Aba2'!$H$498)</f>
+        <v>0.15</v>
+      </c>
+      <c r="D19" s="17">
+        <f>IF((B19+'Aba2'!$F$497+E19)/(1-('Aba2'!$H$497+'Aba1'!$B$17+'Aba1'!$B$18))&lt;'Aba2'!$D$498,'Aba2'!$F$497,'Aba2'!$F$498)</f>
+        <v>6</v>
+      </c>
+      <c r="E19" s="21">
+        <f>'Aba2'!$G$497</f>
+        <v>0</v>
+      </c>
+      <c r="F19" s="9">
+        <f>1-(C19+'Aba1'!$B$17+'Aba1'!$B$18)</f>
+        <v>0.51</v>
+      </c>
+      <c r="G19" s="17">
+        <f>IF(F19&lt;=0,"Ajuste Margem",MAX((B19+D19+E19)/F19,IF(C19='Aba2'!$H$498,'Aba2'!$D$498,0)))</f>
+        <v>171.56862745098039</v>
+      </c>
+      <c r="H19" s="22">
+        <f>G19-(B19+D19+E19+(G19*C19)+(G19*'Aba1'!$B$18))</f>
+        <v>51.470588235294116</v>
+      </c>
+      <c r="I19" s="16">
+        <f>H19/G19</f>
+        <v>0.3</v>
+      </c>
+      <c r="J19" s="17">
+        <f>G19*C19</f>
+        <v>25.735294117647058</v>
+      </c>
+      <c r="K19" s="5"/>
+      <c r="L19" s="18">
+        <f>G19-D19-E19-J19</f>
+        <v>139.83333333333331</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>

</xml_diff>